<commit_message>
Refactor: tach config db services; gioi han rate limit; test API
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/scripts/template_tbqc.xlsx
+++ b/scripts/template_tbqc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aafed2084b17602e/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tbqc\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{718DDFA5-019B-4CF0-A221-CA09247A8C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7811654-AB8F-4493-B3FF-712A6D93FF8A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03A9A2BA-77CE-462A-AC41-CC5884C1C2A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="template" sheetId="1" r:id="rId1"/>
@@ -23,18 +23,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>ID</t>
   </si>
   <si>
     <t>Nhánh</t>
-  </si>
-  <si>
-    <t>P-8-1193</t>
-  </si>
-  <si>
-    <t>Năm</t>
   </si>
 </sst>
 </file>
@@ -383,7 +377,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="16" customWidth="1"/>
@@ -397,14 +391,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>